<commit_message>
correccion 2023 y 2024 y mantener ciertos traits
</commit_message>
<xml_diff>
--- a/NUMEX_pre_RStudio/models_iWUE.xlsx
+++ b/NUMEX_pre_RStudio/models_iWUE.xlsx
@@ -350,7 +350,7 @@
     <t xml:space="preserve">123.5</t>
   </si>
   <si>
-    <t xml:space="preserve">d13C | 1000 | Pouteria</t>
+    <t xml:space="preserve">δ13C | 1000 | Pouteria</t>
   </si>
   <si>
     <t xml:space="preserve">-31.553***</t>
@@ -386,7 +386,7 @@
     <t xml:space="preserve">108.9</t>
   </si>
   <si>
-    <t xml:space="preserve">d13C | 1000 | Clarisia</t>
+    <t xml:space="preserve">δ13C | 1000 | Clarisia</t>
   </si>
   <si>
     <t xml:space="preserve">-30.630***</t>
@@ -419,7 +419,7 @@
     <t xml:space="preserve">35.4</t>
   </si>
   <si>
-    <t xml:space="preserve">d13C | 2000 | Alchornea</t>
+    <t xml:space="preserve">δ13C | 2000 | Alchornea</t>
   </si>
   <si>
     <t xml:space="preserve">-26.513***</t>
@@ -458,7 +458,7 @@
     <t xml:space="preserve">154.2</t>
   </si>
   <si>
-    <t xml:space="preserve">d13C | 2000 | Myrcia</t>
+    <t xml:space="preserve">δ13C | 2000 | Myrcia</t>
   </si>
   <si>
     <t xml:space="preserve">-27.794***</t>
@@ -491,7 +491,7 @@
     <t xml:space="preserve">149.5</t>
   </si>
   <si>
-    <t xml:space="preserve">d13C | 3000 | Hedyosmum</t>
+    <t xml:space="preserve">δ13C | 3000 | Hedyosmum</t>
   </si>
   <si>
     <t xml:space="preserve">-26.806***</t>
@@ -524,7 +524,7 @@
     <t xml:space="preserve">84.3</t>
   </si>
   <si>
-    <t xml:space="preserve">d13C | 3000 | Weinmannia</t>
+    <t xml:space="preserve">δ13C | 3000 | Weinmannia</t>
   </si>
   <si>
     <t xml:space="preserve">-27.724***</t>

</xml_diff>

<commit_message>
templats para tablas, se trabaja con eemeans el dummies es el mas  importante imagenes generadas etc
</commit_message>
<xml_diff>
--- a/NUMEX_pre_RStudio/models_iWUE.xlsx
+++ b/NUMEX_pre_RStudio/models_iWUE.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="241" uniqueCount="241">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="247" uniqueCount="247">
   <si>
     <t xml:space="preserve">Modelo</t>
   </si>
@@ -65,13 +65,13 @@
     <t xml:space="preserve">(Intercept)</t>
   </si>
   <si>
-    <t xml:space="preserve">SUBN</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SUBNP</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SUBP</t>
+    <t xml:space="preserve">N</t>
+  </si>
+  <si>
+    <t xml:space="preserve">P</t>
+  </si>
+  <si>
+    <t xml:space="preserve">N × P</t>
   </si>
   <si>
     <t xml:space="preserve">SD (Intercept Bloque)</t>
@@ -119,18 +119,18 @@
     <t xml:space="preserve">(6.899)</t>
   </si>
   <si>
-    <t xml:space="preserve">-2.266</t>
-  </si>
-  <si>
-    <t xml:space="preserve">(7.634)</t>
-  </si>
-  <si>
     <t xml:space="preserve">3.507</t>
   </si>
   <si>
     <t xml:space="preserve">(7.336)</t>
   </si>
   <si>
+    <t xml:space="preserve">-20.319+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(10.694)</t>
+  </si>
+  <si>
     <t xml:space="preserve">0.000</t>
   </si>
   <si>
@@ -161,13 +161,16 @@
     <t xml:space="preserve">(11.588)</t>
   </si>
   <si>
-    <t xml:space="preserve">-3.011</t>
+    <t xml:space="preserve">9.654</t>
   </si>
   <si>
     <t xml:space="preserve">(7.665)</t>
   </si>
   <si>
-    <t xml:space="preserve">9.654</t>
+    <t xml:space="preserve">1.726</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(13.588)</t>
   </si>
   <si>
     <t xml:space="preserve">10.035</t>
@@ -197,138 +200,141 @@
     <t xml:space="preserve">(6.100)</t>
   </si>
   <si>
-    <t xml:space="preserve">-3.023</t>
+    <t xml:space="preserve">-7.081</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(5.507)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4.022</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(8.734)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">7.244</t>
+  </si>
+  <si>
+    <t xml:space="preserve">14.106</t>
+  </si>
+  <si>
+    <t xml:space="preserve">45</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.039</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.240</t>
+  </si>
+  <si>
+    <t xml:space="preserve">358.9</t>
+  </si>
+  <si>
+    <t xml:space="preserve">iWUE | 2000 | Myrcia</t>
+  </si>
+  <si>
+    <t xml:space="preserve">72.017***</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(3.032)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6.687</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(4.794)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5.608</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(4.548)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-5.984</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(6.714)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">11.743</t>
+  </si>
+  <si>
+    <t xml:space="preserve">50</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.057</t>
+  </si>
+  <si>
+    <t xml:space="preserve">379.2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">iWUE | 3000 | Hedyosmum</t>
+  </si>
+  <si>
+    <t xml:space="preserve">83.754***</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(9.142)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5.492</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(12.379)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-5.891</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(11.970)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">24.202</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(18.768)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">20.443</t>
+  </si>
+  <si>
+    <t xml:space="preserve">21</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.188</t>
+  </si>
+  <si>
+    <t xml:space="preserve">169.3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">iWUE | 3000 | Weinmannia</t>
+  </si>
+  <si>
+    <t xml:space="preserve">72.573***</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(4.962)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-4.231</t>
   </si>
   <si>
     <t xml:space="preserve">(6.485)</t>
   </si>
   <si>
-    <t xml:space="preserve">-7.081</t>
-  </si>
-  <si>
-    <t xml:space="preserve">(5.507)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">7.244</t>
-  </si>
-  <si>
-    <t xml:space="preserve">14.106</t>
-  </si>
-  <si>
-    <t xml:space="preserve">45</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.039</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.240</t>
-  </si>
-  <si>
-    <t xml:space="preserve">358.9</t>
-  </si>
-  <si>
-    <t xml:space="preserve">iWUE | 2000 | Myrcia</t>
-  </si>
-  <si>
-    <t xml:space="preserve">72.017***</t>
-  </si>
-  <si>
-    <t xml:space="preserve">(3.032)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">6.687</t>
-  </si>
-  <si>
-    <t xml:space="preserve">(4.794)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">6.311</t>
-  </si>
-  <si>
-    <t xml:space="preserve">(4.450)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">5.608</t>
-  </si>
-  <si>
-    <t xml:space="preserve">(4.548)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">11.743</t>
-  </si>
-  <si>
-    <t xml:space="preserve">50</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.057</t>
-  </si>
-  <si>
-    <t xml:space="preserve">379.2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">iWUE | 3000 | Hedyosmum</t>
-  </si>
-  <si>
-    <t xml:space="preserve">83.754***</t>
-  </si>
-  <si>
-    <t xml:space="preserve">(9.142)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">5.492</t>
-  </si>
-  <si>
-    <t xml:space="preserve">(12.379)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">23.803</t>
-  </si>
-  <si>
-    <t xml:space="preserve">(14.929)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">-5.891</t>
-  </si>
-  <si>
-    <t xml:space="preserve">(11.970)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">20.443</t>
-  </si>
-  <si>
-    <t xml:space="preserve">21</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.188</t>
-  </si>
-  <si>
-    <t xml:space="preserve">169.3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">iWUE | 3000 | Weinmannia</t>
-  </si>
-  <si>
-    <t xml:space="preserve">72.573***</t>
-  </si>
-  <si>
-    <t xml:space="preserve">(4.962)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">-4.231</t>
-  </si>
-  <si>
-    <t xml:space="preserve">-14.823</t>
-  </si>
-  <si>
-    <t xml:space="preserve">(8.634)</t>
-  </si>
-  <si>
     <t xml:space="preserve">-7.506</t>
   </si>
   <si>
     <t xml:space="preserve">(6.217)</t>
   </si>
   <si>
+    <t xml:space="preserve">-3.086</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(10.545)</t>
+  </si>
+  <si>
     <t xml:space="preserve">3.322</t>
   </si>
   <si>
@@ -347,7 +353,7 @@
     <t xml:space="preserve">123.4</t>
   </si>
   <si>
-    <t xml:space="preserve">d13C | 1000 | Pouteria</t>
+    <t xml:space="preserve">δ13C | 1000 | Pouteria</t>
   </si>
   <si>
     <t xml:space="preserve">-31.553***</t>
@@ -362,18 +368,18 @@
     <t xml:space="preserve">(0.419)</t>
   </si>
   <si>
-    <t xml:space="preserve">-0.183</t>
-  </si>
-  <si>
-    <t xml:space="preserve">(0.464)</t>
-  </si>
-  <si>
     <t xml:space="preserve">0.285</t>
   </si>
   <si>
     <t xml:space="preserve">(0.446)</t>
   </si>
   <si>
+    <t xml:space="preserve">-0.750</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(0.650)</t>
+  </si>
+  <si>
     <t xml:space="preserve">0.960</t>
   </si>
   <si>
@@ -383,7 +389,7 @@
     <t xml:space="preserve">108.9</t>
   </si>
   <si>
-    <t xml:space="preserve">d13C | 1000 | Clarisia</t>
+    <t xml:space="preserve">δ13C | 1000 | Clarisia</t>
   </si>
   <si>
     <t xml:space="preserve">-30.630***</t>
@@ -398,13 +404,16 @@
     <t xml:space="preserve">(0.945)</t>
   </si>
   <si>
-    <t xml:space="preserve">-0.245</t>
+    <t xml:space="preserve">0.788</t>
   </si>
   <si>
     <t xml:space="preserve">(0.625)</t>
   </si>
   <si>
-    <t xml:space="preserve">0.788</t>
+    <t xml:space="preserve">0.138</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(1.108)</t>
   </si>
   <si>
     <t xml:space="preserve">0.818</t>
@@ -416,7 +425,7 @@
     <t xml:space="preserve">35.4</t>
   </si>
   <si>
-    <t xml:space="preserve">d13C | 2000 | Alchornea</t>
+    <t xml:space="preserve">δ13C | 2000 | Alchornea</t>
   </si>
   <si>
     <t xml:space="preserve">-26.513***</t>
@@ -431,18 +440,18 @@
     <t xml:space="preserve">(0.502)</t>
   </si>
   <si>
-    <t xml:space="preserve">-0.244</t>
-  </si>
-  <si>
-    <t xml:space="preserve">(0.534)</t>
-  </si>
-  <si>
     <t xml:space="preserve">-0.581</t>
   </si>
   <si>
     <t xml:space="preserve">(0.453)</t>
   </si>
   <si>
+    <t xml:space="preserve">0.332</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(0.719)</t>
+  </si>
+  <si>
     <t xml:space="preserve">0.598</t>
   </si>
   <si>
@@ -452,7 +461,7 @@
     <t xml:space="preserve">154.2</t>
   </si>
   <si>
-    <t xml:space="preserve">d13C | 2000 | Myrcia</t>
+    <t xml:space="preserve">δ13C | 2000 | Myrcia</t>
   </si>
   <si>
     <t xml:space="preserve">-27.794***</t>
@@ -467,25 +476,25 @@
     <t xml:space="preserve">(0.395)</t>
   </si>
   <si>
-    <t xml:space="preserve">0.522</t>
-  </si>
-  <si>
-    <t xml:space="preserve">(0.366)</t>
-  </si>
-  <si>
     <t xml:space="preserve">0.457</t>
   </si>
   <si>
     <t xml:space="preserve">(0.374)</t>
   </si>
   <si>
+    <t xml:space="preserve">-0.486</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(0.553)</t>
+  </si>
+  <si>
     <t xml:space="preserve">0.966</t>
   </si>
   <si>
     <t xml:space="preserve">149.5</t>
   </si>
   <si>
-    <t xml:space="preserve">d13C | 3000 | Hedyosmum</t>
+    <t xml:space="preserve">δ13C | 3000 | Hedyosmum</t>
   </si>
   <si>
     <t xml:space="preserve">-26.806***</t>
@@ -500,25 +509,25 @@
     <t xml:space="preserve">(1.016)</t>
   </si>
   <si>
-    <t xml:space="preserve">1.956</t>
-  </si>
-  <si>
-    <t xml:space="preserve">(1.225)</t>
-  </si>
-  <si>
     <t xml:space="preserve">-0.483</t>
   </si>
   <si>
     <t xml:space="preserve">(0.982)</t>
   </si>
   <si>
+    <t xml:space="preserve">1.986</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(1.540)</t>
+  </si>
+  <si>
     <t xml:space="preserve">1.677</t>
   </si>
   <si>
     <t xml:space="preserve">84.3</t>
   </si>
   <si>
-    <t xml:space="preserve">d13C | 3000 | Weinmannia</t>
+    <t xml:space="preserve">δ13C | 3000 | Weinmannia</t>
   </si>
   <si>
     <t xml:space="preserve">-27.724***</t>
@@ -533,18 +542,18 @@
     <t xml:space="preserve">(0.531)</t>
   </si>
   <si>
-    <t xml:space="preserve">-1.212</t>
-  </si>
-  <si>
-    <t xml:space="preserve">(0.706)</t>
-  </si>
-  <si>
     <t xml:space="preserve">-0.613</t>
   </si>
   <si>
     <t xml:space="preserve">(0.509)</t>
   </si>
   <si>
+    <t xml:space="preserve">-0.253</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(0.863)</t>
+  </si>
+  <si>
     <t xml:space="preserve">0.272</t>
   </si>
   <si>
@@ -572,43 +581,49 @@
     <t xml:space="preserve">(0.026)</t>
   </si>
   <si>
-    <t xml:space="preserve">0.009</t>
+    <t xml:space="preserve">-0.013</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(0.028)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.077+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(0.041)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.060</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-68.5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ci | 1000 | Clarisia</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.860***</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(0.022)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.055</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(0.044)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-0.037</t>
   </si>
   <si>
     <t xml:space="preserve">(0.029)</t>
   </si>
   <si>
-    <t xml:space="preserve">-0.013</t>
-  </si>
-  <si>
-    <t xml:space="preserve">(0.028)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.060</t>
-  </si>
-  <si>
-    <t xml:space="preserve">-68.5</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ci | 1000 | Clarisia</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.860***</t>
-  </si>
-  <si>
-    <t xml:space="preserve">(0.022)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.055</t>
-  </si>
-  <si>
-    <t xml:space="preserve">(0.044)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.011</t>
-  </si>
-  <si>
-    <t xml:space="preserve">-0.037</t>
+    <t xml:space="preserve">-0.007</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(0.052)</t>
   </si>
   <si>
     <t xml:space="preserve">-13.7</t>
@@ -626,109 +641,112 @@
     <t xml:space="preserve">(0.023)</t>
   </si>
   <si>
+    <t xml:space="preserve">0.027</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-0.015</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(0.033)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.028</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.054</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.238</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-97.7</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ci | 2000 | Myrcia</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.725***</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(0.012)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-0.025</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-0.022</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(0.017)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.023</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.045</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-133.3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ci | 3000 | Hedyosmum</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.682***</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(0.035)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-0.021</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(0.047)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.022</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(0.045)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-0.092</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(0.071)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.078</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-20.2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ci | 3000 | Weinmannia</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.724***</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(0.019)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.016</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(0.025)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.029</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(0.024)</t>
+  </si>
+  <si>
     <t xml:space="preserve">0.012</t>
   </si>
   <si>
-    <t xml:space="preserve">(0.025)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.027</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.028</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.054</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.238</t>
-  </si>
-  <si>
-    <t xml:space="preserve">-97.7</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ci | 2000 | Myrcia</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.725***</t>
-  </si>
-  <si>
-    <t xml:space="preserve">(0.012)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">-0.025</t>
-  </si>
-  <si>
-    <t xml:space="preserve">-0.024</t>
-  </si>
-  <si>
-    <t xml:space="preserve">(0.017)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">-0.022</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.045</t>
-  </si>
-  <si>
-    <t xml:space="preserve">-133.3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ci | 3000 | Hedyosmum</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.682***</t>
-  </si>
-  <si>
-    <t xml:space="preserve">(0.035)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">-0.021</t>
-  </si>
-  <si>
-    <t xml:space="preserve">(0.047)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">-0.090</t>
-  </si>
-  <si>
-    <t xml:space="preserve">(0.057)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.022</t>
-  </si>
-  <si>
-    <t xml:space="preserve">(0.045)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.078</t>
-  </si>
-  <si>
-    <t xml:space="preserve">-20.2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ci | 3000 | Weinmannia</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.724***</t>
-  </si>
-  <si>
-    <t xml:space="preserve">(0.019)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.016</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.056</t>
-  </si>
-  <si>
-    <t xml:space="preserve">(0.033)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.029</t>
-  </si>
-  <si>
-    <t xml:space="preserve">(0.024)</t>
+    <t xml:space="preserve">(0.040)</t>
   </si>
   <si>
     <t xml:space="preserve">0.013</t>
@@ -1301,530 +1319,530 @@
         <v>51</v>
       </c>
       <c r="I5" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="J5" t="s">
         <v>39</v>
       </c>
       <c r="K5" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="L5" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="M5" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="N5" t="s">
         <v>29</v>
       </c>
       <c r="O5" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B6" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C6" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D6" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="E6" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="F6" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="G6" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="H6" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="I6" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="J6" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="K6" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="L6" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="M6" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="N6" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="O6" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="B7" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="C7" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="D7" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="E7" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="F7" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="G7" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="H7" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="I7" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="J7" t="s">
         <v>39</v>
       </c>
       <c r="K7" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="L7" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="M7" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="N7" t="s">
         <v>29</v>
       </c>
       <c r="O7" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="B8" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="C8" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="D8" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="E8" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="F8" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="G8" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="H8" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="I8" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="J8" t="s">
         <v>39</v>
       </c>
       <c r="K8" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="L8" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="M8" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="N8" t="s">
         <v>29</v>
       </c>
       <c r="O8" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="B9" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="C9" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="D9" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="E9" t="s">
-        <v>62</v>
+        <v>102</v>
       </c>
       <c r="F9" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="G9" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="H9" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="I9" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="J9" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="K9" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="L9" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="M9" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="N9" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="O9" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="B10" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="C10" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="D10" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="E10" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="F10" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="G10" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="H10" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="I10" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="J10" t="s">
         <v>39</v>
       </c>
       <c r="K10" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="L10" t="s">
         <v>41</v>
       </c>
       <c r="M10" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="N10" t="s">
         <v>29</v>
       </c>
       <c r="O10" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="B11" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="C11" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="D11" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="E11" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="F11" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="G11" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="H11" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="I11" t="s">
-        <v>129</v>
+        <v>133</v>
       </c>
       <c r="J11" t="s">
         <v>39</v>
       </c>
       <c r="K11" t="s">
-        <v>131</v>
+        <v>134</v>
       </c>
       <c r="L11" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="M11" t="s">
-        <v>132</v>
+        <v>135</v>
       </c>
       <c r="N11" t="s">
         <v>29</v>
       </c>
       <c r="O11" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>134</v>
+        <v>137</v>
       </c>
       <c r="B12" t="s">
-        <v>135</v>
+        <v>138</v>
       </c>
       <c r="C12" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
       <c r="D12" t="s">
-        <v>137</v>
+        <v>140</v>
       </c>
       <c r="E12" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="F12" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="G12" t="s">
-        <v>140</v>
+        <v>143</v>
       </c>
       <c r="H12" t="s">
-        <v>141</v>
+        <v>144</v>
       </c>
       <c r="I12" t="s">
-        <v>142</v>
+        <v>145</v>
       </c>
       <c r="J12" t="s">
-        <v>143</v>
+        <v>146</v>
       </c>
       <c r="K12" t="s">
-        <v>144</v>
+        <v>147</v>
       </c>
       <c r="L12" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="M12" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="N12" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="O12" t="s">
-        <v>145</v>
+        <v>148</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
       <c r="B13" t="s">
-        <v>147</v>
+        <v>150</v>
       </c>
       <c r="C13" t="s">
-        <v>148</v>
+        <v>151</v>
       </c>
       <c r="D13" t="s">
-        <v>149</v>
+        <v>152</v>
       </c>
       <c r="E13" t="s">
-        <v>150</v>
+        <v>153</v>
       </c>
       <c r="F13" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
       <c r="G13" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="H13" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
       <c r="I13" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
       <c r="J13" t="s">
         <v>39</v>
       </c>
       <c r="K13" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="L13" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="M13" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="N13" t="s">
         <v>29</v>
       </c>
       <c r="O13" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="B14" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="C14" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="D14" t="s">
-        <v>160</v>
+        <v>163</v>
       </c>
       <c r="E14" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="F14" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="G14" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="H14" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="I14" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="J14" t="s">
         <v>39</v>
       </c>
       <c r="K14" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="L14" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="M14" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="N14" t="s">
         <v>29</v>
       </c>
       <c r="O14" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>168</v>
+        <v>171</v>
       </c>
       <c r="B15" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="C15" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="D15" t="s">
-        <v>171</v>
+        <v>174</v>
       </c>
       <c r="E15" t="s">
-        <v>172</v>
+        <v>175</v>
       </c>
       <c r="F15" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="G15" t="s">
-        <v>174</v>
+        <v>177</v>
       </c>
       <c r="H15" t="s">
-        <v>175</v>
+        <v>178</v>
       </c>
       <c r="I15" t="s">
-        <v>176</v>
+        <v>179</v>
       </c>
       <c r="J15" t="s">
-        <v>177</v>
+        <v>180</v>
       </c>
       <c r="K15" t="s">
-        <v>178</v>
+        <v>181</v>
       </c>
       <c r="L15" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="M15" t="s">
-        <v>179</v>
+        <v>182</v>
       </c>
       <c r="N15" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="O15" t="s">
-        <v>180</v>
+        <v>183</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>181</v>
+        <v>184</v>
       </c>
       <c r="B16" t="s">
-        <v>182</v>
+        <v>185</v>
       </c>
       <c r="C16" t="s">
-        <v>183</v>
+        <v>186</v>
       </c>
       <c r="D16" t="s">
-        <v>184</v>
+        <v>187</v>
       </c>
       <c r="E16" t="s">
-        <v>185</v>
+        <v>188</v>
       </c>
       <c r="F16" t="s">
-        <v>186</v>
+        <v>189</v>
       </c>
       <c r="G16" t="s">
-        <v>187</v>
+        <v>190</v>
       </c>
       <c r="H16" t="s">
-        <v>188</v>
+        <v>191</v>
       </c>
       <c r="I16" t="s">
-        <v>189</v>
+        <v>192</v>
       </c>
       <c r="J16" t="s">
         <v>39</v>
       </c>
       <c r="K16" t="s">
-        <v>190</v>
+        <v>193</v>
       </c>
       <c r="L16" t="s">
         <v>41</v>
@@ -1836,242 +1854,242 @@
         <v>29</v>
       </c>
       <c r="O16" t="s">
-        <v>191</v>
+        <v>194</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>192</v>
+        <v>195</v>
       </c>
       <c r="B17" t="s">
-        <v>193</v>
+        <v>196</v>
       </c>
       <c r="C17" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
       <c r="D17" t="s">
-        <v>195</v>
+        <v>198</v>
       </c>
       <c r="E17" t="s">
-        <v>196</v>
+        <v>199</v>
       </c>
       <c r="F17" t="s">
-        <v>197</v>
+        <v>200</v>
       </c>
       <c r="G17" t="s">
-        <v>187</v>
+        <v>201</v>
       </c>
       <c r="H17" t="s">
-        <v>198</v>
+        <v>202</v>
       </c>
       <c r="I17" t="s">
-        <v>187</v>
+        <v>203</v>
       </c>
       <c r="J17" t="s">
         <v>39</v>
       </c>
       <c r="K17" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="L17" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="M17" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="N17" t="s">
         <v>29</v>
       </c>
       <c r="O17" t="s">
-        <v>199</v>
+        <v>204</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>200</v>
+        <v>205</v>
       </c>
       <c r="B18" t="s">
-        <v>201</v>
+        <v>206</v>
       </c>
       <c r="C18" t="s">
-        <v>202</v>
+        <v>207</v>
       </c>
       <c r="D18" t="s">
         <v>39</v>
       </c>
       <c r="E18" t="s">
-        <v>203</v>
+        <v>208</v>
       </c>
       <c r="F18" t="s">
-        <v>204</v>
+        <v>209</v>
       </c>
       <c r="G18" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="H18" t="s">
-        <v>206</v>
+        <v>210</v>
       </c>
       <c r="I18" t="s">
-        <v>202</v>
+        <v>211</v>
       </c>
       <c r="J18" t="s">
-        <v>207</v>
+        <v>212</v>
       </c>
       <c r="K18" t="s">
-        <v>208</v>
+        <v>213</v>
       </c>
       <c r="L18" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="M18" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="N18" t="s">
-        <v>209</v>
+        <v>214</v>
       </c>
       <c r="O18" t="s">
-        <v>210</v>
+        <v>215</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>211</v>
+        <v>216</v>
       </c>
       <c r="B19" t="s">
-        <v>212</v>
+        <v>217</v>
       </c>
       <c r="C19" t="s">
-        <v>213</v>
+        <v>218</v>
       </c>
       <c r="D19" t="s">
-        <v>214</v>
+        <v>219</v>
       </c>
       <c r="E19" t="s">
-        <v>183</v>
+        <v>186</v>
       </c>
       <c r="F19" t="s">
-        <v>215</v>
+        <v>220</v>
       </c>
       <c r="G19" t="s">
-        <v>216</v>
+        <v>221</v>
       </c>
       <c r="H19" t="s">
-        <v>217</v>
+        <v>222</v>
       </c>
       <c r="I19" t="s">
-        <v>216</v>
+        <v>188</v>
       </c>
       <c r="J19" t="s">
         <v>39</v>
       </c>
       <c r="K19" t="s">
-        <v>218</v>
+        <v>223</v>
       </c>
       <c r="L19" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="M19" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="N19" t="s">
         <v>29</v>
       </c>
       <c r="O19" t="s">
-        <v>219</v>
+        <v>224</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>220</v>
+        <v>225</v>
       </c>
       <c r="B20" t="s">
-        <v>221</v>
+        <v>226</v>
       </c>
       <c r="C20" t="s">
-        <v>222</v>
+        <v>227</v>
       </c>
       <c r="D20" t="s">
-        <v>223</v>
+        <v>228</v>
       </c>
       <c r="E20" t="s">
-        <v>224</v>
+        <v>229</v>
       </c>
       <c r="F20" t="s">
-        <v>225</v>
+        <v>230</v>
       </c>
       <c r="G20" t="s">
-        <v>226</v>
+        <v>231</v>
       </c>
       <c r="H20" t="s">
-        <v>227</v>
+        <v>232</v>
       </c>
       <c r="I20" t="s">
-        <v>228</v>
+        <v>233</v>
       </c>
       <c r="J20" t="s">
         <v>39</v>
       </c>
       <c r="K20" t="s">
-        <v>229</v>
+        <v>234</v>
       </c>
       <c r="L20" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="M20" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="N20" t="s">
         <v>29</v>
       </c>
       <c r="O20" t="s">
-        <v>230</v>
+        <v>235</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="s">
-        <v>231</v>
+        <v>236</v>
       </c>
       <c r="B21" t="s">
-        <v>232</v>
+        <v>237</v>
       </c>
       <c r="C21" t="s">
-        <v>233</v>
+        <v>238</v>
       </c>
       <c r="D21" t="s">
-        <v>234</v>
+        <v>239</v>
       </c>
       <c r="E21" t="s">
-        <v>205</v>
+        <v>240</v>
       </c>
       <c r="F21" t="s">
-        <v>235</v>
+        <v>241</v>
       </c>
       <c r="G21" t="s">
-        <v>236</v>
+        <v>242</v>
       </c>
       <c r="H21" t="s">
-        <v>237</v>
+        <v>243</v>
       </c>
       <c r="I21" t="s">
-        <v>238</v>
+        <v>244</v>
       </c>
       <c r="J21" t="s">
-        <v>239</v>
+        <v>245</v>
       </c>
       <c r="K21" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="L21" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="M21" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="N21" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="O21" t="s">
-        <v>240</v>
+        <v>246</v>
       </c>
     </row>
   </sheetData>

</xml_diff>